<commit_message>
Added state options to each @ngxs state. Also moved models over to libraries
</commit_message>
<xml_diff>
--- a/apps/assets-firefly/docs/release-schedule.xlsx
+++ b/apps/assets-firefly/docs/release-schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andredavcev/Projects/theory/apps/assets-firefly/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93A33D33-047F-C242-B162-E52DC226A302}" xr6:coauthVersionLast="38" xr6:coauthVersionMax="38" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2460AB48-462A-EF45-B6DD-660C0179E33C}" xr6:coauthVersionLast="38" xr6:coauthVersionMax="38" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1500" yWindow="560" windowWidth="22720" windowHeight="18820" xr2:uid="{D9A7F54E-A8DF-8F44-8DA3-CE45AC6D884A}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="75">
   <si>
     <t>Version</t>
   </si>
@@ -244,6 +244,12 @@
   </si>
   <si>
     <t>Network State/Base Component</t>
+  </si>
+  <si>
+    <t>Friends</t>
+  </si>
+  <si>
+    <t>Event/Location/Subscription Chats</t>
   </si>
 </sst>
 </file>
@@ -605,7 +611,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E808F83-7B39-7A4C-8F08-E0AB4C8C7AD2}">
-  <dimension ref="B2:F51"/>
+  <dimension ref="B2:F53"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2.6640625" customWidth="1"/>
@@ -914,36 +920,46 @@
     </row>
     <row r="48" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B48" t="s">
-        <v>25</v>
-      </c>
-      <c r="C48" t="s">
-        <v>16</v>
+        <v>73</v>
       </c>
     </row>
     <row r="49" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B49" t="s">
-        <v>52</v>
+        <v>25</v>
       </c>
       <c r="C49" t="s">
-        <v>53</v>
+        <v>16</v>
       </c>
     </row>
     <row r="50" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B50" t="s">
-        <v>55</v>
-      </c>
-      <c r="C50" t="s">
-        <v>54</v>
-      </c>
-      <c r="D50" t="s">
-        <v>58</v>
+        <v>74</v>
       </c>
     </row>
     <row r="51" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B51" t="s">
+        <v>52</v>
+      </c>
+      <c r="C51" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="52" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B52" t="s">
+        <v>55</v>
+      </c>
+      <c r="C52" t="s">
+        <v>54</v>
+      </c>
+      <c r="D52" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="53" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B53" t="s">
         <v>57</v>
       </c>
-      <c r="C51" t="s">
+      <c r="C53" t="s">
         <v>59</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Updated all local paths to @firefly/core, @firefly/mobile, @firefly/app, & @firefly/env
</commit_message>
<xml_diff>
--- a/apps/assets-firefly/docs/release-schedule.xlsx
+++ b/apps/assets-firefly/docs/release-schedule.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andredavcev/Projects/theory/apps/assets-firefly/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2460AB48-462A-EF45-B6DD-660C0179E33C}" xr6:coauthVersionLast="38" xr6:coauthVersionMax="38" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3671EEBF-20E9-6645-9117-99A0D0C047E3}" xr6:coauthVersionLast="38" xr6:coauthVersionMax="38" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1500" yWindow="560" windowWidth="22720" windowHeight="18820" xr2:uid="{D9A7F54E-A8DF-8F44-8DA3-CE45AC6D884A}"/>
+    <workbookView xWindow="540" yWindow="480" windowWidth="22720" windowHeight="18820" xr2:uid="{D9A7F54E-A8DF-8F44-8DA3-CE45AC6D884A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="77">
   <si>
     <t>Version</t>
   </si>
@@ -250,6 +250,12 @@
   </si>
   <si>
     <t>Event/Location/Subscription Chats</t>
+  </si>
+  <si>
+    <t>Splash Screen</t>
+  </si>
+  <si>
+    <t>App Icon</t>
   </si>
 </sst>
 </file>
@@ -611,7 +617,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E808F83-7B39-7A4C-8F08-E0AB4C8C7AD2}">
-  <dimension ref="B2:F53"/>
+  <dimension ref="B2:F55"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2.6640625" customWidth="1"/>
@@ -761,205 +767,215 @@
     </row>
     <row r="24" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B24" t="s">
-        <v>45</v>
-      </c>
-      <c r="C24" t="s">
-        <v>7</v>
-      </c>
-      <c r="D24" t="s">
-        <v>47</v>
+        <v>75</v>
       </c>
     </row>
     <row r="25" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B25" t="s">
-        <v>27</v>
-      </c>
-      <c r="D25" t="s">
-        <v>46</v>
+        <v>76</v>
       </c>
     </row>
     <row r="26" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B26" t="s">
-        <v>28</v>
+        <v>45</v>
+      </c>
+      <c r="C26" t="s">
+        <v>7</v>
+      </c>
+      <c r="D26" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="27" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B27" t="s">
-        <v>32</v>
+        <v>27</v>
+      </c>
+      <c r="D27" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="28" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B28" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
     </row>
     <row r="29" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B29" t="s">
-        <v>40</v>
+        <v>32</v>
       </c>
     </row>
     <row r="30" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B30" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
     </row>
     <row r="31" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B31" t="s">
-        <v>62</v>
+        <v>40</v>
       </c>
     </row>
     <row r="32" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B32" t="s">
-        <v>63</v>
+        <v>41</v>
       </c>
     </row>
     <row r="33" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B33" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
     </row>
     <row r="34" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B34" t="s">
-        <v>72</v>
+        <v>63</v>
       </c>
     </row>
     <row r="35" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B35" t="s">
-        <v>17</v>
-      </c>
-      <c r="C35" t="s">
-        <v>8</v>
-      </c>
-      <c r="D35" t="s">
-        <v>31</v>
+        <v>65</v>
       </c>
     </row>
     <row r="36" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B36" t="s">
-        <v>50</v>
+        <v>72</v>
       </c>
     </row>
     <row r="37" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B37" t="s">
-        <v>29</v>
+        <v>17</v>
+      </c>
+      <c r="C37" t="s">
+        <v>8</v>
+      </c>
+      <c r="D37" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="38" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B38" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="39" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B39" t="s">
-        <v>18</v>
-      </c>
-      <c r="C39" t="s">
-        <v>9</v>
+        <v>29</v>
       </c>
     </row>
     <row r="40" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B40" t="s">
-        <v>64</v>
+        <v>48</v>
       </c>
     </row>
     <row r="41" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B41" t="s">
-        <v>66</v>
+        <v>18</v>
+      </c>
+      <c r="C41" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="42" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B42" t="s">
-        <v>19</v>
-      </c>
-      <c r="C42" t="s">
-        <v>10</v>
-      </c>
-      <c r="D42" t="s">
-        <v>49</v>
+        <v>64</v>
       </c>
     </row>
     <row r="43" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B43" t="s">
-        <v>20</v>
-      </c>
-      <c r="C43" t="s">
-        <v>11</v>
+        <v>66</v>
       </c>
     </row>
     <row r="44" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B44" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C44" t="s">
-        <v>12</v>
+        <v>10</v>
+      </c>
+      <c r="D44" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="45" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B45" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C45" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="46" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B46" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C46" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="47" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B47" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C47" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="48" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B48" t="s">
-        <v>73</v>
+        <v>23</v>
+      </c>
+      <c r="C48" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="49" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B49" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C49" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="50" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B50" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="51" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B51" t="s">
-        <v>52</v>
+        <v>25</v>
       </c>
       <c r="C51" t="s">
-        <v>53</v>
+        <v>16</v>
       </c>
     </row>
     <row r="52" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B52" t="s">
-        <v>55</v>
-      </c>
-      <c r="C52" t="s">
-        <v>54</v>
-      </c>
-      <c r="D52" t="s">
-        <v>58</v>
+        <v>74</v>
       </c>
     </row>
     <row r="53" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B53" t="s">
+        <v>52</v>
+      </c>
+      <c r="C53" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="54" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B54" t="s">
+        <v>55</v>
+      </c>
+      <c r="C54" t="s">
+        <v>54</v>
+      </c>
+      <c r="D54" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="55" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B55" t="s">
         <v>57</v>
       </c>
-      <c r="C53" t="s">
+      <c r="C55" t="s">
         <v>59</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Start of functions-firefly refactor. Changed tslint.json & tsconfig.json
</commit_message>
<xml_diff>
--- a/apps/assets-firefly/docs/release-schedule.xlsx
+++ b/apps/assets-firefly/docs/release-schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andredavcev/Projects/theory/apps/assets-firefly/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3671EEBF-20E9-6645-9117-99A0D0C047E3}" xr6:coauthVersionLast="38" xr6:coauthVersionMax="38" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E0D6339-A54E-5D4F-BB6C-7C9EC14EF443}" xr6:coauthVersionLast="38" xr6:coauthVersionMax="38" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="540" yWindow="480" windowWidth="22720" windowHeight="18820" xr2:uid="{D9A7F54E-A8DF-8F44-8DA3-CE45AC6D884A}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="78">
   <si>
     <t>Version</t>
   </si>
@@ -256,6 +256,9 @@
   </si>
   <si>
     <t>App Icon</t>
+  </si>
+  <si>
+    <t>Input Border Directive</t>
   </si>
 </sst>
 </file>
@@ -617,7 +620,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E808F83-7B39-7A4C-8F08-E0AB4C8C7AD2}">
-  <dimension ref="B2:F55"/>
+  <dimension ref="B2:F56"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2.6640625" customWidth="1"/>
@@ -719,263 +722,268 @@
     </row>
     <row r="15" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B15" t="s">
-        <v>58</v>
-      </c>
-      <c r="C15" t="s">
-        <v>6</v>
+        <v>77</v>
       </c>
     </row>
     <row r="16" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B16" t="s">
-        <v>30</v>
+        <v>58</v>
+      </c>
+      <c r="C16" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B17" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
     </row>
     <row r="18" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B18" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="19" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B19" t="s">
-        <v>51</v>
+        <v>37</v>
       </c>
     </row>
     <row r="20" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B20" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
     </row>
     <row r="21" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B21" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="22" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B22" t="s">
-        <v>56</v>
+        <v>39</v>
       </c>
     </row>
     <row r="23" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B23" t="s">
-        <v>68</v>
+        <v>56</v>
       </c>
     </row>
     <row r="24" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B24" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
     </row>
     <row r="25" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B25" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="26" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B26" t="s">
-        <v>45</v>
-      </c>
-      <c r="C26" t="s">
-        <v>7</v>
-      </c>
-      <c r="D26" t="s">
-        <v>47</v>
+        <v>76</v>
       </c>
     </row>
     <row r="27" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B27" t="s">
-        <v>27</v>
+        <v>45</v>
+      </c>
+      <c r="C27" t="s">
+        <v>7</v>
       </c>
       <c r="D27" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="28" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B28" t="s">
-        <v>28</v>
+        <v>27</v>
+      </c>
+      <c r="D28" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="29" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B29" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
     </row>
     <row r="30" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B30" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="31" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B31" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
     </row>
     <row r="32" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B32" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="33" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B33" t="s">
-        <v>62</v>
+        <v>41</v>
       </c>
     </row>
     <row r="34" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B34" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="35" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B35" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="36" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B36" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
     </row>
     <row r="37" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B37" t="s">
-        <v>17</v>
-      </c>
-      <c r="C37" t="s">
-        <v>8</v>
-      </c>
-      <c r="D37" t="s">
-        <v>31</v>
+        <v>72</v>
       </c>
     </row>
     <row r="38" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B38" t="s">
-        <v>50</v>
+        <v>17</v>
+      </c>
+      <c r="C38" t="s">
+        <v>8</v>
+      </c>
+      <c r="D38" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="39" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B39" t="s">
-        <v>29</v>
+        <v>50</v>
       </c>
     </row>
     <row r="40" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B40" t="s">
-        <v>48</v>
+        <v>29</v>
       </c>
     </row>
     <row r="41" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B41" t="s">
-        <v>18</v>
-      </c>
-      <c r="C41" t="s">
-        <v>9</v>
+        <v>48</v>
       </c>
     </row>
     <row r="42" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B42" t="s">
-        <v>64</v>
+        <v>18</v>
+      </c>
+      <c r="C42" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="43" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B43" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="44" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B44" t="s">
-        <v>19</v>
-      </c>
-      <c r="C44" t="s">
-        <v>10</v>
-      </c>
-      <c r="D44" t="s">
-        <v>49</v>
+        <v>66</v>
       </c>
     </row>
     <row r="45" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B45" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C45" t="s">
-        <v>11</v>
+        <v>10</v>
+      </c>
+      <c r="D45" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="46" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B46" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C46" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="47" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B47" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C47" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="48" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B48" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C48" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="49" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B49" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C49" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="50" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B50" t="s">
-        <v>73</v>
+        <v>24</v>
+      </c>
+      <c r="C50" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="51" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B51" t="s">
-        <v>25</v>
-      </c>
-      <c r="C51" t="s">
-        <v>16</v>
+        <v>73</v>
       </c>
     </row>
     <row r="52" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B52" t="s">
-        <v>74</v>
+        <v>25</v>
+      </c>
+      <c r="C52" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="53" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B53" t="s">
-        <v>52</v>
-      </c>
-      <c r="C53" t="s">
-        <v>53</v>
+        <v>74</v>
       </c>
     </row>
     <row r="54" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B54" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="C54" t="s">
-        <v>54</v>
-      </c>
-      <c r="D54" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
     </row>
     <row r="55" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B55" t="s">
+        <v>55</v>
+      </c>
+      <c r="C55" t="s">
+        <v>54</v>
+      </c>
+      <c r="D55" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="56" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B56" t="s">
         <v>57</v>
       </c>
-      <c r="C55" t="s">
+      <c r="C56" t="s">
         <v>59</v>
       </c>
     </row>

</xml_diff>